<commit_message>
APR refresh P-0→P-6: ignition audit + DAILY Aug10-12 append + marginal logger init
- P-0: APR multi-chain (ETH/BSC/Monad), no CEX spot; BSC DEX vol $42.6M/day
- P-1: 3 rows appended CASE_APR.xlsx DAILY (Oct23→Aug12, 294 rows)
  Aug12: c=$0.607, vol=$903M (+192.3%), NEW ATH HIGH intraday $0.6325
- P-2: CẦN OPERATOR (Nansen LOCKED, BSC contract 0x299ad4... confirmed)
- P-3: GOM-D 4/4 PASS, suppressor OFF, Aug12 vol-wake 345× — draft chưa ký
- P-4: hedge_struct OFF toàn bộ Aug05-12, div_avg3 BULL 1.6-1.9 — không mode-switch
- P-5: Aug12 = SHORT SQUEEZE (OI+6.5% vs vol 345×), gLSR rising 0.97→1.33 BULL
- P-6: 5/5 PASS (row count, date continuity, no neg close, Aug12 pump, taker range)
- data/logs/marginal_hits.csv: khởi tạo header — MARGINAL-V4 logger sẵn sàng
- .gitignore: thêm !data/logs/ exception (force-add)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_APR.xlsx
+++ b/docs/case_files/CASE_APR.xlsx
@@ -798,7 +798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX293"/>
+  <dimension ref="A1:AX296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42701,6 +42701,402 @@
         <is>
           <t>false</t>
         </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>0.1967333333333333</v>
+      </c>
+      <c r="C294" t="n">
+        <v>0.1992</v>
+      </c>
+      <c r="D294" t="n">
+        <v>0.2034</v>
+      </c>
+      <c r="E294" t="n">
+        <v>0.1891</v>
+      </c>
+      <c r="F294" t="n">
+        <v>0.1977</v>
+      </c>
+      <c r="G294" t="n">
+        <v>1940969.2344</v>
+      </c>
+      <c r="H294" t="n">
+        <v>48.65836742084942</v>
+      </c>
+      <c r="I294" t="n">
+        <v>0.0002637483333333333</v>
+      </c>
+      <c r="J294" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="K294" t="n">
+        <v>0.00050001</v>
+      </c>
+      <c r="L294" t="n">
+        <v>6</v>
+      </c>
+      <c r="M294" t="n">
+        <v>9271101.8532</v>
+      </c>
+      <c r="N294" t="n">
+        <v>46565052</v>
+      </c>
+      <c r="O294" t="n">
+        <v>1</v>
+      </c>
+      <c r="P294" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q294" t="n">
+        <v>-0.7031642390758475</v>
+      </c>
+      <c r="R294" t="n">
+        <v>0</v>
+      </c>
+      <c r="S294" t="n">
+        <v>0</v>
+      </c>
+      <c r="T294" t="n">
+        <v>1.043545329259211</v>
+      </c>
+      <c r="U294" t="n">
+        <v>0.719854330288357</v>
+      </c>
+      <c r="V294" t="n">
+        <v>2.131170973062122</v>
+      </c>
+      <c r="X294" t="n">
+        <v>0.8287160133802213</v>
+      </c>
+      <c r="Y294" t="n">
+        <v>3.541666666666656</v>
+      </c>
+      <c r="Z294" t="n">
+        <v>-21.4594127806563</v>
+      </c>
+      <c r="AA294" t="n">
+        <v>1.9383</v>
+      </c>
+      <c r="AB294" t="n">
+        <v>0.9095</v>
+      </c>
+      <c r="AC294" t="n">
+        <v>0.9661999999999999</v>
+      </c>
+      <c r="AD294" t="n">
+        <v>0.9491000000000001</v>
+      </c>
+      <c r="AK294" t="inlineStr">
+        <is>
+          <t>CoinGecko/BSC+ETH+Monad</t>
+        </is>
+      </c>
+      <c r="AO294" t="inlineStr">
+        <is>
+          <t>fapi.binance.com klines 1d</t>
+        </is>
+      </c>
+      <c r="AP294" t="inlineStr">
+        <is>
+          <t>fapi.binance.com topPos/topAcc/global/taker</t>
+        </is>
+      </c>
+      <c r="AQ294" t="n">
+        <v>0.3793651697184734</v>
+      </c>
+      <c r="AR294" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS294" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT294" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU294" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV294" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW294" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX294" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>0.2039666666666667</v>
+      </c>
+      <c r="C295" t="n">
+        <v>0.1976</v>
+      </c>
+      <c r="D295" t="n">
+        <v>0.2079</v>
+      </c>
+      <c r="E295" t="n">
+        <v>0.1962</v>
+      </c>
+      <c r="F295" t="n">
+        <v>0.2078</v>
+      </c>
+      <c r="G295" t="n">
+        <v>1965766.9715</v>
+      </c>
+      <c r="H295" t="n">
+        <v>47.98321707889169</v>
+      </c>
+      <c r="I295" t="n">
+        <v>0.000130415</v>
+      </c>
+      <c r="J295" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="K295" t="n">
+        <v>0.00033548</v>
+      </c>
+      <c r="L295" t="n">
+        <v>6</v>
+      </c>
+      <c r="M295" t="n">
+        <v>9095395.372033499</v>
+      </c>
+      <c r="N295" t="n">
+        <v>46019070</v>
+      </c>
+      <c r="O295" t="n">
+        <v>1</v>
+      </c>
+      <c r="P295" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q295" t="n">
+        <v>5.108750632271131</v>
+      </c>
+      <c r="R295" t="n">
+        <v>0</v>
+      </c>
+      <c r="S295" t="n">
+        <v>0</v>
+      </c>
+      <c r="T295" t="n">
+        <v>1.023767995276133</v>
+      </c>
+      <c r="U295" t="n">
+        <v>0.7520151736142805</v>
+      </c>
+      <c r="V295" t="n">
+        <v>1.557080220850926</v>
+      </c>
+      <c r="W295" t="n">
+        <v>1.800943440287703</v>
+      </c>
+      <c r="X295" t="n">
+        <v>1.255536454646577</v>
+      </c>
+      <c r="Y295" t="n">
+        <v>-1.062786978279934</v>
+      </c>
+      <c r="Z295" t="n">
+        <v>35.41506322155031</v>
+      </c>
+      <c r="AA295" t="n">
+        <v>1.9177</v>
+      </c>
+      <c r="AB295" t="n">
+        <v>1.2316</v>
+      </c>
+      <c r="AC295" t="n">
+        <v>1.2416</v>
+      </c>
+      <c r="AD295" t="n">
+        <v>0.9226</v>
+      </c>
+      <c r="AK295" t="inlineStr">
+        <is>
+          <t>CoinGecko/BSC+ETH+Monad</t>
+        </is>
+      </c>
+      <c r="AO295" t="inlineStr">
+        <is>
+          <t>fapi.binance.com klines 1d</t>
+        </is>
+      </c>
+      <c r="AP295" t="inlineStr">
+        <is>
+          <t>fapi.binance.com topPos/topAcc/global/taker</t>
+        </is>
+      </c>
+      <c r="AQ295" t="n">
+        <v>0.3133809525063222</v>
+      </c>
+      <c r="AR295" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS295" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT295" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU295" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV295" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW295" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX295" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>0.4822333333333333</v>
+      </c>
+      <c r="C296" t="n">
+        <v>0.2076</v>
+      </c>
+      <c r="D296" t="n">
+        <v>0.6325</v>
+      </c>
+      <c r="E296" t="n">
+        <v>0.2068</v>
+      </c>
+      <c r="F296" t="n">
+        <v>0.6074000000000001</v>
+      </c>
+      <c r="G296" t="n">
+        <v>903339470.6586699</v>
+      </c>
+      <c r="H296" t="n">
+        <v>51.95693523323135</v>
+      </c>
+      <c r="I296" t="n">
+        <v>0.0002265583333333333</v>
+      </c>
+      <c r="J296" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="K296" t="n">
+        <v>0.00060334</v>
+      </c>
+      <c r="L296" t="n">
+        <v>6</v>
+      </c>
+      <c r="M296" t="n">
+        <v>9689917.191729</v>
+      </c>
+      <c r="N296" t="n">
+        <v>46642515</v>
+      </c>
+      <c r="O296" t="n">
+        <v>1</v>
+      </c>
+      <c r="P296" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q296" t="n">
+        <v>192.3002887391723</v>
+      </c>
+      <c r="R296" t="n">
+        <v>0</v>
+      </c>
+      <c r="S296" t="n">
+        <v>0</v>
+      </c>
+      <c r="T296" t="n">
+        <v>1.090686736749325</v>
+      </c>
+      <c r="U296" t="n">
+        <v>345.5775779677718</v>
+      </c>
+      <c r="V296" t="n">
+        <v>1.498530463102709</v>
+      </c>
+      <c r="W296" t="n">
+        <v>1.688970588235294</v>
+      </c>
+      <c r="X296" t="n">
+        <v>1.122109158186864</v>
+      </c>
+      <c r="Y296" t="n">
+        <v>-2.672444925966045</v>
+      </c>
+      <c r="Z296" t="n">
+        <v>38.41671247938427</v>
+      </c>
+      <c r="AA296" t="n">
+        <v>1.8865</v>
+      </c>
+      <c r="AB296" t="n">
+        <v>1.2589</v>
+      </c>
+      <c r="AC296" t="n">
+        <v>1.3343</v>
+      </c>
+      <c r="AD296" t="n">
+        <v>1.0745</v>
+      </c>
+      <c r="AK296" t="inlineStr">
+        <is>
+          <t>CoinGecko/BSC+ETH+Monad</t>
+        </is>
+      </c>
+      <c r="AO296" t="inlineStr">
+        <is>
+          <t>fapi.binance.com klines 1d</t>
+        </is>
+      </c>
+      <c r="AP296" t="inlineStr">
+        <is>
+          <t>fapi.binance.com topPos/topAcc/global/taker</t>
+        </is>
+      </c>
+      <c r="AQ296" t="n">
+        <v>0.5366456643582297</v>
+      </c>
+      <c r="AR296" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS296" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT296" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU296" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV296" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW296" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX296" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
spot-venue patch S0-S6: AIN/GUA=binance_alpha, APR=kucoin (wash flag)
- Venue discovery: AIN/GUA/APR đều WASH trên top CEX (31x/196x/98x)
- AIN+GUA override → binance_alpha (store sạch hơn MEXC wash)
- APR: kucoin win (1.51M/day), BSC DEX negligible ($758)
- col31/32/33 filled: GUA 40r + APR 43r (CASE_AIN locked → temp file)
- AIN exit: 739d@10% Alpha vol — effectively illiquid
- GUA vol spike Aug05-11: +397% với price giảm — distribution signal
- APR claim $42.6M/day vs KuCoin thực 1.51M = 28x off

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_APR.xlsx
+++ b/docs/case_files/CASE_APR.xlsx
@@ -36438,9 +36438,11 @@
       <c r="AD254" s="14" t="n">
         <v>0.9496550973326324</v>
       </c>
-      <c r="AE254" s="14" t="inlineStr"/>
-      <c r="AF254" s="14" t="inlineStr"/>
-      <c r="AG254" s="14" t="inlineStr"/>
+      <c r="AE254" s="14" t="n">
+        <v>120860.37</v>
+      </c>
+      <c r="AF254" s="14" t="n"/>
+      <c r="AG254" s="14" t="n"/>
       <c r="AH254" s="14" t="inlineStr"/>
       <c r="AI254" s="14" t="inlineStr">
         <is>
@@ -36594,9 +36596,11 @@
       <c r="AD255" s="14" t="n">
         <v>0.8142457120034781</v>
       </c>
-      <c r="AE255" s="14" t="inlineStr"/>
-      <c r="AF255" s="14" t="inlineStr"/>
-      <c r="AG255" s="14" t="inlineStr"/>
+      <c r="AE255" s="14" t="n">
+        <v>98680.88</v>
+      </c>
+      <c r="AF255" s="14" t="n"/>
+      <c r="AG255" s="14" t="n"/>
       <c r="AH255" s="14" t="inlineStr"/>
       <c r="AI255" s="14" t="inlineStr">
         <is>
@@ -36750,9 +36754,11 @@
       <c r="AD256" s="14" t="n">
         <v>0.9584829397650404</v>
       </c>
-      <c r="AE256" s="14" t="inlineStr"/>
-      <c r="AF256" s="14" t="inlineStr"/>
-      <c r="AG256" s="14" t="inlineStr"/>
+      <c r="AE256" s="14" t="n">
+        <v>43791.69</v>
+      </c>
+      <c r="AF256" s="14" t="n"/>
+      <c r="AG256" s="14" t="n"/>
       <c r="AH256" s="14" t="inlineStr"/>
       <c r="AI256" s="14" t="inlineStr">
         <is>
@@ -36906,9 +36912,11 @@
       <c r="AD257" s="14" t="n">
         <v>0.8590722824294629</v>
       </c>
-      <c r="AE257" s="14" t="inlineStr"/>
-      <c r="AF257" s="14" t="inlineStr"/>
-      <c r="AG257" s="14" t="inlineStr"/>
+      <c r="AE257" s="14" t="n">
+        <v>20825.05</v>
+      </c>
+      <c r="AF257" s="14" t="n"/>
+      <c r="AG257" s="14" t="n"/>
       <c r="AH257" s="14" t="inlineStr"/>
       <c r="AI257" s="14" t="inlineStr">
         <is>
@@ -37062,9 +37070,11 @@
       <c r="AD258" s="14" t="n">
         <v>1.07634354892753</v>
       </c>
-      <c r="AE258" s="14" t="inlineStr"/>
-      <c r="AF258" s="14" t="inlineStr"/>
-      <c r="AG258" s="14" t="inlineStr"/>
+      <c r="AE258" s="14" t="n">
+        <v>72029.92</v>
+      </c>
+      <c r="AF258" s="14" t="n"/>
+      <c r="AG258" s="14" t="n"/>
       <c r="AH258" s="14" t="inlineStr"/>
       <c r="AI258" s="14" t="inlineStr">
         <is>
@@ -37222,9 +37232,11 @@
       <c r="AD259" s="14" t="n">
         <v>0.9344021074234776</v>
       </c>
-      <c r="AE259" s="14" t="inlineStr"/>
-      <c r="AF259" s="14" t="inlineStr"/>
-      <c r="AG259" s="14" t="inlineStr"/>
+      <c r="AE259" s="14" t="n">
+        <v>46588.05</v>
+      </c>
+      <c r="AF259" s="14" t="n"/>
+      <c r="AG259" s="14" t="n"/>
       <c r="AH259" s="14" t="inlineStr"/>
       <c r="AI259" s="14" t="inlineStr">
         <is>
@@ -37378,9 +37390,11 @@
       <c r="AD260" s="14" t="n">
         <v>0.9753367267882268</v>
       </c>
-      <c r="AE260" s="14" t="inlineStr"/>
-      <c r="AF260" s="14" t="inlineStr"/>
-      <c r="AG260" s="14" t="inlineStr"/>
+      <c r="AE260" s="14" t="n">
+        <v>36660.16</v>
+      </c>
+      <c r="AF260" s="14" t="n"/>
+      <c r="AG260" s="14" t="n"/>
       <c r="AH260" s="14" t="inlineStr"/>
       <c r="AI260" s="14" t="inlineStr">
         <is>
@@ -37534,9 +37548,11 @@
       <c r="AD261" s="14" t="n">
         <v>0.949664800041624</v>
       </c>
-      <c r="AE261" s="14" t="inlineStr"/>
-      <c r="AF261" s="14" t="inlineStr"/>
-      <c r="AG261" s="14" t="inlineStr"/>
+      <c r="AE261" s="14" t="n">
+        <v>42527.9</v>
+      </c>
+      <c r="AF261" s="14" t="n"/>
+      <c r="AG261" s="14" t="n"/>
       <c r="AH261" s="14" t="inlineStr"/>
       <c r="AI261" s="14" t="inlineStr">
         <is>
@@ -37690,9 +37706,11 @@
       <c r="AD262" s="14" t="n">
         <v>0.8166694113025433</v>
       </c>
-      <c r="AE262" s="14" t="inlineStr"/>
-      <c r="AF262" s="14" t="inlineStr"/>
-      <c r="AG262" s="14" t="inlineStr"/>
+      <c r="AE262" s="14" t="n">
+        <v>18799.51</v>
+      </c>
+      <c r="AF262" s="14" t="n"/>
+      <c r="AG262" s="14" t="n"/>
       <c r="AH262" s="14" t="inlineStr"/>
       <c r="AI262" s="14" t="inlineStr">
         <is>
@@ -37846,9 +37864,11 @@
       <c r="AD263" s="14" t="n">
         <v>1.059999680578949</v>
       </c>
-      <c r="AE263" s="14" t="inlineStr"/>
-      <c r="AF263" s="14" t="inlineStr"/>
-      <c r="AG263" s="14" t="inlineStr"/>
+      <c r="AE263" s="14" t="n">
+        <v>17036.21</v>
+      </c>
+      <c r="AF263" s="14" t="n"/>
+      <c r="AG263" s="14" t="n"/>
       <c r="AH263" s="14" t="inlineStr"/>
       <c r="AI263" s="14" t="inlineStr">
         <is>
@@ -38002,9 +38022,11 @@
       <c r="AD264" s="14" t="n">
         <v>0.9419084735050482</v>
       </c>
-      <c r="AE264" s="14" t="inlineStr"/>
-      <c r="AF264" s="14" t="inlineStr"/>
-      <c r="AG264" s="14" t="inlineStr"/>
+      <c r="AE264" s="14" t="n">
+        <v>61301.97</v>
+      </c>
+      <c r="AF264" s="14" t="n"/>
+      <c r="AG264" s="14" t="n"/>
       <c r="AH264" s="14" t="inlineStr"/>
       <c r="AI264" s="14" t="inlineStr">
         <is>
@@ -38162,9 +38184,13 @@
       <c r="AD265" s="14" t="n">
         <v>1.027488323272699</v>
       </c>
-      <c r="AE265" s="14" t="inlineStr"/>
-      <c r="AF265" s="14" t="inlineStr"/>
-      <c r="AG265" s="14" t="inlineStr"/>
+      <c r="AE265" s="14" t="n">
+        <v>30678.18</v>
+      </c>
+      <c r="AF265" s="14" t="n"/>
+      <c r="AG265" s="14" t="n">
+        <v>0.003231</v>
+      </c>
       <c r="AH265" s="14" t="inlineStr"/>
       <c r="AI265" s="14" t="inlineStr">
         <is>
@@ -38322,9 +38348,13 @@
       <c r="AD266" s="14" t="n">
         <v>0.905838599867248</v>
       </c>
-      <c r="AE266" s="14" t="inlineStr"/>
-      <c r="AF266" s="14" t="inlineStr"/>
-      <c r="AG266" s="14" t="inlineStr"/>
+      <c r="AE266" s="14" t="n">
+        <v>53610.76</v>
+      </c>
+      <c r="AF266" s="14" t="n"/>
+      <c r="AG266" s="14" t="n">
+        <v>0.005216</v>
+      </c>
       <c r="AH266" s="14" t="inlineStr"/>
       <c r="AI266" s="14" t="inlineStr">
         <is>
@@ -38482,9 +38512,13 @@
       <c r="AD267" s="14" t="n">
         <v>0.9635347183991276</v>
       </c>
-      <c r="AE267" s="14" t="inlineStr"/>
-      <c r="AF267" s="14" t="inlineStr"/>
-      <c r="AG267" s="14" t="inlineStr"/>
+      <c r="AE267" s="14" t="n">
+        <v>63867.37</v>
+      </c>
+      <c r="AF267" s="14" t="n"/>
+      <c r="AG267" s="14" t="n">
+        <v>0.0068</v>
+      </c>
       <c r="AH267" s="14" t="inlineStr"/>
       <c r="AI267" s="14" t="inlineStr">
         <is>
@@ -38642,9 +38676,13 @@
       <c r="AD268" s="14" t="n">
         <v>0.9605577222110836</v>
       </c>
-      <c r="AE268" s="14" t="inlineStr"/>
-      <c r="AF268" s="14" t="inlineStr"/>
-      <c r="AG268" s="14" t="inlineStr"/>
+      <c r="AE268" s="14" t="n">
+        <v>47367.93</v>
+      </c>
+      <c r="AF268" s="14" t="n"/>
+      <c r="AG268" s="14" t="n">
+        <v>0.00501</v>
+      </c>
       <c r="AH268" s="14" t="inlineStr"/>
       <c r="AI268" s="14" t="inlineStr">
         <is>
@@ -38802,9 +38840,13 @@
       <c r="AD269" s="14" t="n">
         <v>1.200131229264558</v>
       </c>
-      <c r="AE269" s="14" t="inlineStr"/>
-      <c r="AF269" s="14" t="inlineStr"/>
-      <c r="AG269" s="14" t="inlineStr"/>
+      <c r="AE269" s="14" t="n">
+        <v>34199.73</v>
+      </c>
+      <c r="AF269" s="14" t="n"/>
+      <c r="AG269" s="14" t="n">
+        <v>0.003629</v>
+      </c>
       <c r="AH269" s="14" t="inlineStr"/>
       <c r="AI269" s="14" t="inlineStr">
         <is>
@@ -38962,9 +39004,13 @@
       <c r="AD270" s="14" t="n">
         <v>0.9868165960607348</v>
       </c>
-      <c r="AE270" s="14" t="inlineStr"/>
-      <c r="AF270" s="14" t="inlineStr"/>
-      <c r="AG270" s="14" t="inlineStr"/>
+      <c r="AE270" s="14" t="n">
+        <v>40192.76</v>
+      </c>
+      <c r="AF270" s="14" t="n"/>
+      <c r="AG270" s="14" t="n">
+        <v>0.004135</v>
+      </c>
       <c r="AH270" s="14" t="inlineStr"/>
       <c r="AI270" s="14" t="inlineStr">
         <is>
@@ -39122,9 +39168,13 @@
       <c r="AD271" s="14" t="n">
         <v>1.013091468576515</v>
       </c>
-      <c r="AE271" s="14" t="inlineStr"/>
-      <c r="AF271" s="14" t="inlineStr"/>
-      <c r="AG271" s="14" t="inlineStr"/>
+      <c r="AE271" s="14" t="n">
+        <v>23984.96</v>
+      </c>
+      <c r="AF271" s="14" t="n"/>
+      <c r="AG271" s="14" t="n">
+        <v>0.002558</v>
+      </c>
       <c r="AH271" s="14" t="inlineStr"/>
       <c r="AI271" s="14" t="inlineStr">
         <is>
@@ -39284,9 +39334,13 @@
       <c r="AD272" s="14" t="n">
         <v>0.85381705643743</v>
       </c>
-      <c r="AE272" s="14" t="inlineStr"/>
-      <c r="AF272" s="14" t="inlineStr"/>
-      <c r="AG272" s="14" t="inlineStr"/>
+      <c r="AE272" s="14" t="n">
+        <v>38075.58</v>
+      </c>
+      <c r="AF272" s="14" t="n"/>
+      <c r="AG272" s="14" t="n">
+        <v>0.003959</v>
+      </c>
       <c r="AH272" s="14" t="inlineStr"/>
       <c r="AI272" s="14" t="inlineStr">
         <is>
@@ -39446,9 +39500,13 @@
       <c r="AD273" s="14" t="n">
         <v>0.9158730737407392</v>
       </c>
-      <c r="AE273" s="14" t="inlineStr"/>
-      <c r="AF273" s="14" t="inlineStr"/>
-      <c r="AG273" s="14" t="inlineStr"/>
+      <c r="AE273" s="14" t="n">
+        <v>16946.91</v>
+      </c>
+      <c r="AF273" s="14" t="n"/>
+      <c r="AG273" s="14" t="n">
+        <v>0.001776</v>
+      </c>
       <c r="AH273" s="14" t="inlineStr"/>
       <c r="AI273" s="14" t="inlineStr">
         <is>
@@ -39608,9 +39666,13 @@
       <c r="AD274" s="14" t="n">
         <v>0.8756275490872794</v>
       </c>
-      <c r="AE274" s="14" t="inlineStr"/>
-      <c r="AF274" s="14" t="inlineStr"/>
-      <c r="AG274" s="14" t="inlineStr"/>
+      <c r="AE274" s="14" t="n">
+        <v>29644.95</v>
+      </c>
+      <c r="AF274" s="14" t="n"/>
+      <c r="AG274" s="14" t="n">
+        <v>0.003132</v>
+      </c>
       <c r="AH274" s="14" t="inlineStr"/>
       <c r="AI274" s="14" t="inlineStr">
         <is>
@@ -39772,9 +39834,13 @@
       <c r="AD275" s="14" t="n">
         <v>0.7407839683808324</v>
       </c>
-      <c r="AE275" s="14" t="inlineStr"/>
-      <c r="AF275" s="14" t="inlineStr"/>
-      <c r="AG275" s="14" t="inlineStr"/>
+      <c r="AE275" s="14" t="n">
+        <v>21265.7</v>
+      </c>
+      <c r="AF275" s="14" t="n"/>
+      <c r="AG275" s="14" t="n">
+        <v>0.002266</v>
+      </c>
       <c r="AH275" s="14" t="inlineStr"/>
       <c r="AI275" s="14" t="inlineStr">
         <is>
@@ -39936,9 +40002,13 @@
       <c r="AD276" s="14" t="n">
         <v>0.9041377382073656</v>
       </c>
-      <c r="AE276" s="14" t="inlineStr"/>
-      <c r="AF276" s="14" t="inlineStr"/>
-      <c r="AG276" s="14" t="inlineStr"/>
+      <c r="AE276" s="14" t="n">
+        <v>108217.22</v>
+      </c>
+      <c r="AF276" s="14" t="n"/>
+      <c r="AG276" s="14" t="n">
+        <v>0.012025</v>
+      </c>
       <c r="AH276" s="14" t="inlineStr"/>
       <c r="AI276" s="14" t="inlineStr">
         <is>
@@ -40082,9 +40152,13 @@
       <c r="AB277" s="14" t="inlineStr"/>
       <c r="AC277" s="14" t="inlineStr"/>
       <c r="AD277" s="14" t="inlineStr"/>
-      <c r="AE277" s="14" t="inlineStr"/>
-      <c r="AF277" s="14" t="inlineStr"/>
-      <c r="AG277" s="14" t="inlineStr"/>
+      <c r="AE277" s="14" t="n">
+        <v>134453.78</v>
+      </c>
+      <c r="AF277" s="14" t="n"/>
+      <c r="AG277" s="14" t="n">
+        <v>0.014809</v>
+      </c>
       <c r="AH277" s="14" t="inlineStr"/>
       <c r="AI277" s="14" t="inlineStr">
         <is>
@@ -40228,9 +40302,13 @@
       <c r="AB278" s="14" t="inlineStr"/>
       <c r="AC278" s="14" t="inlineStr"/>
       <c r="AD278" s="14" t="inlineStr"/>
-      <c r="AE278" s="14" t="inlineStr"/>
-      <c r="AF278" s="14" t="inlineStr"/>
-      <c r="AG278" s="14" t="inlineStr"/>
+      <c r="AE278" s="14" t="n">
+        <v>57224.83</v>
+      </c>
+      <c r="AF278" s="14" t="n"/>
+      <c r="AG278" s="14" t="n">
+        <v>0.006043</v>
+      </c>
       <c r="AH278" s="14" t="inlineStr"/>
       <c r="AI278" s="14" t="inlineStr">
         <is>
@@ -40374,9 +40452,13 @@
       <c r="AB279" s="14" t="inlineStr"/>
       <c r="AC279" s="14" t="inlineStr"/>
       <c r="AD279" s="14" t="inlineStr"/>
-      <c r="AE279" s="14" t="inlineStr"/>
-      <c r="AF279" s="14" t="inlineStr"/>
-      <c r="AG279" s="14" t="inlineStr"/>
+      <c r="AE279" s="14" t="n">
+        <v>34551.04</v>
+      </c>
+      <c r="AF279" s="14" t="n"/>
+      <c r="AG279" s="14" t="n">
+        <v>0.003725</v>
+      </c>
       <c r="AH279" s="14" t="inlineStr"/>
       <c r="AI279" s="14" t="inlineStr">
         <is>
@@ -40532,9 +40614,13 @@
       <c r="AD280" s="14" t="n">
         <v>0.8628</v>
       </c>
-      <c r="AE280" s="14" t="inlineStr"/>
-      <c r="AF280" s="14" t="inlineStr"/>
-      <c r="AG280" s="14" t="inlineStr"/>
+      <c r="AE280" s="14" t="n">
+        <v>43854.05</v>
+      </c>
+      <c r="AF280" s="14" t="n"/>
+      <c r="AG280" s="14" t="n">
+        <v>0.004853</v>
+      </c>
       <c r="AH280" s="14" t="inlineStr"/>
       <c r="AI280" s="14" t="inlineStr">
         <is>
@@ -40690,9 +40776,13 @@
       <c r="AD281" s="14" t="n">
         <v>0.9897</v>
       </c>
-      <c r="AE281" s="14" t="inlineStr"/>
-      <c r="AF281" s="14" t="inlineStr"/>
-      <c r="AG281" s="14" t="inlineStr"/>
+      <c r="AE281" s="14" t="n">
+        <v>31952.26</v>
+      </c>
+      <c r="AF281" s="14" t="n"/>
+      <c r="AG281" s="14" t="n">
+        <v>0.003559</v>
+      </c>
       <c r="AH281" s="14" t="inlineStr"/>
       <c r="AI281" s="14" t="inlineStr">
         <is>
@@ -40848,9 +40938,13 @@
       <c r="AD282" s="14" t="n">
         <v>0.9313</v>
       </c>
-      <c r="AE282" s="14" t="inlineStr"/>
-      <c r="AF282" s="14" t="inlineStr"/>
-      <c r="AG282" s="14" t="inlineStr"/>
+      <c r="AE282" s="14" t="n">
+        <v>32456.37</v>
+      </c>
+      <c r="AF282" s="14" t="n"/>
+      <c r="AG282" s="14" t="n">
+        <v>0.003691</v>
+      </c>
       <c r="AH282" s="14" t="inlineStr"/>
       <c r="AI282" s="14" t="inlineStr">
         <is>
@@ -41010,9 +41104,13 @@
       <c r="AD283" s="14" t="n">
         <v>1.0004</v>
       </c>
-      <c r="AE283" s="14" t="inlineStr"/>
-      <c r="AF283" s="14" t="inlineStr"/>
-      <c r="AG283" s="14" t="inlineStr"/>
+      <c r="AE283" s="14" t="n">
+        <v>16646.09</v>
+      </c>
+      <c r="AF283" s="14" t="n"/>
+      <c r="AG283" s="14" t="n">
+        <v>0.001869</v>
+      </c>
       <c r="AH283" s="14" t="inlineStr"/>
       <c r="AI283" s="14" t="inlineStr">
         <is>
@@ -41176,9 +41274,13 @@
       <c r="AD284" s="14" t="n">
         <v>1.0206</v>
       </c>
-      <c r="AE284" s="14" t="inlineStr"/>
-      <c r="AF284" s="14" t="inlineStr"/>
-      <c r="AG284" s="14" t="inlineStr"/>
+      <c r="AE284" s="14" t="n">
+        <v>19251.05</v>
+      </c>
+      <c r="AF284" s="14" t="n"/>
+      <c r="AG284" s="14" t="n">
+        <v>0.002188</v>
+      </c>
       <c r="AH284" s="14" t="inlineStr"/>
       <c r="AI284" s="14" t="inlineStr">
         <is>
@@ -41340,9 +41442,13 @@
       <c r="AD285" s="14" t="n">
         <v>0.9828</v>
       </c>
-      <c r="AE285" s="14" t="inlineStr"/>
-      <c r="AF285" s="14" t="inlineStr"/>
-      <c r="AG285" s="14" t="inlineStr"/>
+      <c r="AE285" s="14" t="n">
+        <v>37908.68</v>
+      </c>
+      <c r="AF285" s="14" t="n"/>
+      <c r="AG285" s="14" t="n">
+        <v>0.004278</v>
+      </c>
       <c r="AH285" s="14" t="inlineStr"/>
       <c r="AI285" s="14" t="inlineStr">
         <is>
@@ -41504,9 +41610,13 @@
       <c r="AD286" s="14" t="n">
         <v>0.9375</v>
       </c>
-      <c r="AE286" s="14" t="inlineStr"/>
-      <c r="AF286" s="14" t="inlineStr"/>
-      <c r="AG286" s="14" t="inlineStr"/>
+      <c r="AE286" s="14" t="n">
+        <v>56878.22</v>
+      </c>
+      <c r="AF286" s="14" t="n"/>
+      <c r="AG286" s="14" t="n">
+        <v>0.005207</v>
+      </c>
       <c r="AH286" s="14" t="inlineStr"/>
       <c r="AI286" s="14" t="inlineStr">
         <is>
@@ -41668,9 +41778,13 @@
       <c r="AD287" s="14" t="n">
         <v>1.0287</v>
       </c>
-      <c r="AE287" s="14" t="inlineStr"/>
-      <c r="AF287" s="14" t="inlineStr"/>
-      <c r="AG287" s="14" t="inlineStr"/>
+      <c r="AE287" s="14" t="n">
+        <v>21515.26</v>
+      </c>
+      <c r="AF287" s="14" t="n"/>
+      <c r="AG287" s="14" t="n">
+        <v>0.002311</v>
+      </c>
       <c r="AH287" s="14" t="inlineStr"/>
       <c r="AI287" s="14" t="inlineStr">
         <is>
@@ -41836,9 +41950,13 @@
       <c r="AD288" s="14" t="n">
         <v>0.924</v>
       </c>
-      <c r="AE288" s="14" t="inlineStr"/>
-      <c r="AF288" s="14" t="inlineStr"/>
-      <c r="AG288" s="14" t="inlineStr"/>
+      <c r="AE288" s="14" t="n">
+        <v>16216.17</v>
+      </c>
+      <c r="AF288" s="14" t="n"/>
+      <c r="AG288" s="14" t="n">
+        <v>0.001838</v>
+      </c>
       <c r="AH288" s="14" t="inlineStr"/>
       <c r="AI288" s="14" t="inlineStr">
         <is>
@@ -42000,9 +42118,13 @@
       <c r="AD289" s="14" t="n">
         <v>0.9426</v>
       </c>
-      <c r="AE289" s="14" t="inlineStr"/>
-      <c r="AF289" s="14" t="inlineStr"/>
-      <c r="AG289" s="14" t="inlineStr"/>
+      <c r="AE289" s="14" t="n">
+        <v>29733.33</v>
+      </c>
+      <c r="AF289" s="14" t="n"/>
+      <c r="AG289" s="14" t="n">
+        <v>0.003599</v>
+      </c>
       <c r="AH289" s="14" t="inlineStr"/>
       <c r="AI289" s="14" t="inlineStr">
         <is>
@@ -42168,9 +42290,13 @@
       <c r="AD290" s="14" t="n">
         <v>1.0982</v>
       </c>
-      <c r="AE290" s="14" t="inlineStr"/>
-      <c r="AF290" s="14" t="inlineStr"/>
-      <c r="AG290" s="14" t="inlineStr"/>
+      <c r="AE290" s="14" t="n">
+        <v>50220.07</v>
+      </c>
+      <c r="AF290" s="14" t="n"/>
+      <c r="AG290" s="14" t="n">
+        <v>0.005714</v>
+      </c>
       <c r="AH290" s="14" t="inlineStr"/>
       <c r="AI290" s="14" t="inlineStr">
         <is>
@@ -42340,9 +42466,13 @@
       <c r="AD291" s="14" t="n">
         <v>1.0413</v>
       </c>
-      <c r="AE291" s="14" t="inlineStr"/>
-      <c r="AF291" s="14" t="inlineStr"/>
-      <c r="AG291" s="14" t="inlineStr"/>
+      <c r="AE291" s="14" t="n">
+        <v>75229.63</v>
+      </c>
+      <c r="AF291" s="14" t="n"/>
+      <c r="AG291" s="14" t="n">
+        <v>0.008500000000000001</v>
+      </c>
       <c r="AH291" s="14" t="inlineStr"/>
       <c r="AI291" s="14" t="inlineStr">
         <is>
@@ -42486,9 +42616,13 @@
       <c r="AB292" s="14" t="inlineStr"/>
       <c r="AC292" s="14" t="inlineStr"/>
       <c r="AD292" s="14" t="inlineStr"/>
-      <c r="AE292" s="14" t="inlineStr"/>
-      <c r="AF292" s="14" t="inlineStr"/>
-      <c r="AG292" s="14" t="inlineStr"/>
+      <c r="AE292" s="14" t="n">
+        <v>49569.36</v>
+      </c>
+      <c r="AF292" s="14" t="n"/>
+      <c r="AG292" s="14" t="n">
+        <v>0.004976</v>
+      </c>
       <c r="AH292" s="14" t="inlineStr"/>
       <c r="AI292" s="14" t="inlineStr">
         <is>
@@ -42632,9 +42766,13 @@
       <c r="AB293" s="14" t="inlineStr"/>
       <c r="AC293" s="14" t="inlineStr"/>
       <c r="AD293" s="14" t="inlineStr"/>
-      <c r="AE293" s="14" t="inlineStr"/>
-      <c r="AF293" s="14" t="inlineStr"/>
-      <c r="AG293" s="14" t="inlineStr"/>
+      <c r="AE293" s="14" t="n">
+        <v>71923.63</v>
+      </c>
+      <c r="AF293" s="14" t="n"/>
+      <c r="AG293" s="14" t="n">
+        <v>0.007432</v>
+      </c>
       <c r="AH293" s="14" t="inlineStr"/>
       <c r="AI293" s="14" t="inlineStr">
         <is>
@@ -42793,6 +42931,12 @@
       <c r="AD294" t="n">
         <v>0.9491000000000001</v>
       </c>
+      <c r="AE294" t="n">
+        <v>31251.84</v>
+      </c>
+      <c r="AG294" t="n">
+        <v>0.003371</v>
+      </c>
       <c r="AK294" t="inlineStr">
         <is>
           <t>CoinGecko/BSC+ETH+Monad</t>
@@ -42926,6 +43070,12 @@
       <c r="AD295" t="n">
         <v>0.9226</v>
       </c>
+      <c r="AE295" t="n">
+        <v>26487.55</v>
+      </c>
+      <c r="AG295" t="n">
+        <v>0.002912</v>
+      </c>
       <c r="AK295" t="inlineStr">
         <is>
           <t>CoinGecko/BSC+ETH+Monad</t>
@@ -43058,6 +43208,12 @@
       </c>
       <c r="AD296" t="n">
         <v>1.0745</v>
+      </c>
+      <c r="AE296" t="n">
+        <v>3928680.4</v>
+      </c>
+      <c r="AG296" t="n">
+        <v>0.40544</v>
       </c>
       <c r="AK296" t="inlineStr">
         <is>

</xml_diff>